<commit_message>
test: record reviewed ordinary race and standalone S01-A evidence
</commit_message>
<xml_diff>
--- a/evidence/independent_sample_1.xlsx
+++ b/evidence/independent_sample_1.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>34e67e8adcd9f7bb5c5e4064840591ce</t>
+    <t>97d437b1b685434f96d29496d47ffeae</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>ff38a7be07e24ce1c0d810f9c9d17a51</t>
+    <t>66e17dd00ea230d5c64d9f29841e0a66</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-26T14:13:18+08:00</t>
+    <t>2026-10-26T14:26:19+08:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>